<commit_message>
Update with latest work: V2 methodology, scoring, dashboards and data
- Add PCAF V2 methodology docs (FR/EN) and glossary
- Add V2 livrables: updated scoring, Looker data, dashboards
- Reorganise méthodologie/ with V1 subfolder for legacy docs
- Update analysis results and all Looker CSVs
- Add generate_pcaf_assessment.py and generate_all_looker_csvs.py
- Add Julius Baer 2025 extracted report
- Add feedback files and translation outputs
- Remove livrables/.DS_Store from tracking

Co-Authored-By: Oz <oz-agent@warp.dev>
</commit_message>
<xml_diff>
--- a/livrables/coverage/pcaf_quantile_analysis_FR.xlsx
+++ b/livrables/coverage/pcaf_quantile_analysis_FR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fidestra922-my.sharepoint.com/personal/epl_fidestra922_onmicrosoft_com/Documents/03_ACCOUNTS/Axylia/pcaf-compliance/analysis/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fidestra922-my.sharepoint.com/personal/epl_fidestra922_onmicrosoft_com/Documents/03_ACCOUNTS/Axylia/pcaf-compliance/livrables/coverage/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="20" documentId="11_08526D471F0A5C4851B14C735A2A93BF7BC97F96" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A896616B-A68B-CD42-8FB5-AC9802A8ED98}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="21700" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Matrice de classification" sheetId="1" r:id="rId1"/>

</xml_diff>